<commit_message>
still digging out of the test hell
</commit_message>
<xml_diff>
--- a/ci-cd-merge-resolver/repoCollector/datasets/skywalking.xlsx
+++ b/ci-cd-merge-resolver/repoCollector/datasets/skywalking.xlsx
@@ -192,7 +192,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="n" s="0">
-        <v>0.6269999742507935</v>
+        <v>0.6480000019073486</v>
       </c>
       <c r="J2" t="b" s="0">
         <v>1</v>
@@ -224,7 +224,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="n" s="0">
-        <v>1.1519999504089355</v>
+        <v>1.2680000066757202</v>
       </c>
       <c r="J3" t="b" s="0">
         <v>1</v>
@@ -256,7 +256,7 @@
         <v>1</v>
       </c>
       <c r="I4" t="n" s="0">
-        <v>1.180999994277954</v>
+        <v>0.8040000200271606</v>
       </c>
       <c r="J4" t="b" s="0">
         <v>1</v>
@@ -288,7 +288,7 @@
         <v>1</v>
       </c>
       <c r="I5" t="n" s="0">
-        <v>33.79800033569336</v>
+        <v>33.23699951171875</v>
       </c>
       <c r="J5" t="b" s="0">
         <v>1</v>
@@ -320,7 +320,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="n" s="0">
-        <v>34.05599594116211</v>
+        <v>33.65899658203125</v>
       </c>
       <c r="J6" t="b" s="0">
         <v>1</v>

</xml_diff>

<commit_message>
only four failing tests
</commit_message>
<xml_diff>
--- a/ci-cd-merge-resolver/repoCollector/datasets/skywalking.xlsx
+++ b/ci-cd-merge-resolver/repoCollector/datasets/skywalking.xlsx
@@ -192,7 +192,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="n" s="0">
-        <v>0.7549999952316284</v>
+        <v>0.5270000100135803</v>
       </c>
       <c r="J2" t="b" s="0">
         <v>1</v>
@@ -224,7 +224,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="n" s="0">
-        <v>1.340000033378601</v>
+        <v>1.3170000314712524</v>
       </c>
       <c r="J3" t="b" s="0">
         <v>1</v>
@@ -256,7 +256,7 @@
         <v>1</v>
       </c>
       <c r="I4" t="n" s="0">
-        <v>0.5519999861717224</v>
+        <v>1.4170000553131104</v>
       </c>
       <c r="J4" t="b" s="0">
         <v>1</v>
@@ -288,7 +288,7 @@
         <v>1</v>
       </c>
       <c r="I5" t="n" s="0">
-        <v>37.722999572753906</v>
+        <v>33.53799819946289</v>
       </c>
       <c r="J5" t="b" s="0">
         <v>1</v>
@@ -320,7 +320,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="n" s="0">
-        <v>38.05099868774414</v>
+        <v>34.26899719238281</v>
       </c>
       <c r="J6" t="b" s="0">
         <v>1</v>

</xml_diff>